<commit_message>
daily auto-refresh 2026-08-19 14:22
</commit_message>
<xml_diff>
--- a/segment_monthly.xlsx
+++ b/segment_monthly.xlsx
@@ -987,7 +987,7 @@
         <v>4973</v>
       </c>
       <c r="J13" t="n">
-        <v>40917</v>
+        <v>41074</v>
       </c>
       <c r="K13" t="n">
         <v>12140</v>
@@ -996,7 +996,7 @@
         <v>291915</v>
       </c>
       <c r="M13" t="n">
-        <v>519595</v>
+        <v>519752</v>
       </c>
     </row>
     <row r="14">
@@ -1006,40 +1006,40 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>637</v>
+        <v>661</v>
       </c>
       <c r="C14" t="n">
-        <v>667</v>
+        <v>700</v>
       </c>
       <c r="D14" t="n">
-        <v>48.8</v>
+        <v>48.6</v>
       </c>
       <c r="E14" t="n">
-        <v>840</v>
+        <v>870</v>
       </c>
       <c r="F14" t="n">
-        <v>1029</v>
+        <v>1097</v>
       </c>
       <c r="G14" t="n">
-        <v>974</v>
+        <v>1005</v>
       </c>
       <c r="H14" t="n">
-        <v>1213</v>
+        <v>1287</v>
       </c>
       <c r="I14" t="n">
-        <v>1403</v>
+        <v>1632</v>
       </c>
       <c r="J14" t="n">
-        <v>40288</v>
+        <v>43396</v>
       </c>
       <c r="K14" t="n">
-        <v>12777</v>
+        <v>12801</v>
       </c>
       <c r="L14" t="n">
-        <v>293318</v>
+        <v>293547</v>
       </c>
       <c r="M14" t="n">
-        <v>559883</v>
+        <v>563148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>